<commit_message>
Correccion de datos, ventanas y decision de integracion de las variables endogenas.
</commit_message>
<xml_diff>
--- a/outputs/resultados_johansen.xlsx
+++ b/outputs/resultados_johansen.xlsx
@@ -482,31 +482,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>218</v>
+        <v>252</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>0.05</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Rango completo</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Revisar orden de integración</t>
+          <t>VARX en diferencias</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>El rank es igual al número de variables. Esto no es cointegración propiamente dicha; sugiere revisar si las variables en niveles son I(1).</t>
+          <t>No se encontró relación de cointegración.</t>
         </is>
       </c>
     </row>
@@ -583,19 +583,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>43.10561264905771</v>
+        <v>17.66602552179466</v>
       </c>
       <c r="D2" t="n">
-        <v>13.4294</v>
+        <v>16.1619</v>
       </c>
       <c r="E2" t="n">
-        <v>15.4943</v>
+        <v>18.3985</v>
       </c>
       <c r="F2" t="n">
-        <v>19.9349</v>
+        <v>23.1485</v>
       </c>
       <c r="G2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7.231572994805843</v>
+        <v>4.839733136088213</v>
       </c>
       <c r="D3" t="n">
         <v>2.7055</v>
@@ -637,19 +637,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35.87403965425187</v>
+        <v>12.82629238570645</v>
       </c>
       <c r="D4" t="n">
-        <v>12.2971</v>
+        <v>15.0006</v>
       </c>
       <c r="E4" t="n">
-        <v>14.2639</v>
+        <v>17.1481</v>
       </c>
       <c r="F4" t="n">
-        <v>18.52</v>
+        <v>21.7465</v>
       </c>
       <c r="G4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7.231572994805843</v>
+        <v>4.839733136088213</v>
       </c>
       <c r="D5" t="n">
         <v>2.7055</v>
@@ -703,14 +703,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>(0.15302450554731814+0j)</t>
+          <t>(0.050404259158615426+0j)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>(0.03292526839365561+0j)</t>
+          <t>(0.019325866978879273+0j)</t>
         </is>
       </c>
     </row>

</xml_diff>